<commit_message>
docs(backlog): record Sprint 5 merged and review states
</commit_message>
<xml_diff>
--- a/Nhom8_ProductBacklog.xlsx
+++ b/Nhom8_ProductBacklog.xlsx
@@ -289,7 +289,7 @@
     <t>Đã triển khai sớm và merge PR #4 ngày 28/10: check-in bằng mã theo buổi, cửa sổ thời gian, chống lặp; API + Web + 11 integration test. Chờ Sprint Review 3.</t>
   </si>
   <si>
-    <t>Upload/metadata minh chứng theo storage và validation contract của Phú</t>
+    <t>Done (merge PR #7 ngày 30/10): Kiệt làm 30/10, 5 commit (DTO/service, endpoint, test, Web, docs). Phú review: đúng contract, build 0 warning, 94/94 test, thử Web nộp ảnh/mã, tải file, HSSV duyệt/từ chối qua US-21. Lỗi phía Phú (sinh viên không mở được hoạt động đã kết thúc để nộp minh chứng) sửa ở PR #8, merge 30/10. Chờ Sprint Review 3.</t>
   </si>
   <si>
     <t>Đã triển khai sớm và merge PR #5 ngày 28/10: danh sách người tham gia, điểm danh thủ công, xem/duyệt minh chứng; API + Web + 7 integration test. Chờ US-08 để thử duyệt file thật và Sprint Review 3.</t>
@@ -307,13 +307,13 @@
     <t>View/query gợi ý theo score-gap và eligibility đã có</t>
   </si>
   <si>
-    <t>Scoring service, kỳ đánh giá, duyệt một lần và lịch sử điểm</t>
+    <t>Triển khai sớm, merge PR #9 ngày 30/10: kỳ đánh giá (không trùng/chồng thời gian, khóa/mở), sổ điểm một quyết định cho mỗi đăng ký, ghi điểm cho người đủ điều kiện (đã check-in hoặc có minh chứng được duyệt), lịch sử phê duyệt, khóa điểm danh/minh chứng sau khi ghi điểm; API + Web + 8 test (104/104). Khai báo sẵn chuyển trạng thái cho US-23 của Kiệt.</t>
   </si>
   <si>
     <t>Các transition Reject/Pending/Revoke có lý do theo state machine</t>
   </si>
   <si>
-    <t>Định nghĩa mẫu số/tỷ lệ và API báo cáo tổng hợp, nguy cơ thiếu điểm</t>
+    <t>Triển khai sớm, merge PR #10 ngày 30/10: báo cáo theo kỳ (tổng hợp, từng hoạt động, sinh viên nguy cơ thiếu điểm), lọc theo cơ sở/khóa/lớp, chia theo lớp/khóa/cơ sở; định nghĩa chỉ số ghi trong README (tỷ lệ = tham gia/đăng ký còn hiệu lực, điểm = bản ghi Approved của US-22, nguy cơ = dưới điểm mục tiêu của kỳ). API + Web + 2 test (106/106).</t>
   </si>
   <si>
     <t>Sprint 5</t>
@@ -363,7 +363,7 @@
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="dd\-mmm\-yy"/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="40">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -455,11 +455,6 @@
       <color rgb="FF0000D4"/>
       <name val="Arial"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1182,19 +1177,22 @@
   </borders>
   <cellStyleXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="44" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="41" fontId="16" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="16" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="19" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0">
@@ -1203,148 +1201,142 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="21">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="7" borderId="22">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="23">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="8" borderId="22">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="9" borderId="24">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="25">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="26">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="14" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="16" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="17" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="25" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="28" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="33" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="35" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="36" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="21">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="7" borderId="22">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="23">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="22">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="9" borderId="24">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="25">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="26">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="18" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="22" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="38" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="20">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="20">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="20">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="39" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="40" borderId="19">
+    <xf numFmtId="0" fontId="39" fillId="39" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="40" borderId="19">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1366,9 +1358,6 @@
     </xf>
     <xf numFmtId="176" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1971,12 +1960,12 @@
   <sheetFormatPr defaultColWidth="8.86363636363636" defaultRowHeight="12.5"/>
   <sheetData>
     <row r="2" ht="12.75" customHeight="1" spans="1:1">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="49" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="12" customHeight="1" spans="1:1">
-      <c r="A3" s="52" t="s">
+      <c r="A3" s="50" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2019,109 +2008,109 @@
   </cols>
   <sheetData>
     <row r="1" ht="12.75" customHeight="1" spans="1:6">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="42" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="3" ht="12.75" customHeight="1" spans="1:6">
-      <c r="A3" s="45" t="s">
+      <c r="A3" s="43" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="45" t="s">
+      <c r="B3" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="45" t="s">
+      <c r="C3" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="45" t="s">
+      <c r="E3" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="45" t="s">
+      <c r="F3" s="43" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" ht="12" customHeight="1" spans="1:6">
-      <c r="A4" s="46">
+      <c r="A4" s="44">
         <v>1</v>
       </c>
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="47" t="s">
+      <c r="C4" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="46" t="s">
+      <c r="D4" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="48">
+      <c r="E4" s="46">
         <v>46275</v>
       </c>
-      <c r="F4" s="48">
+      <c r="F4" s="46">
         <v>46383</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1" spans="1:6">
-      <c r="A5" s="46">
+      <c r="A5" s="44">
         <v>2</v>
       </c>
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="44" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="49" t="s">
+      <c r="C5" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="D5" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="48">
+      <c r="E5" s="46">
         <v>46275</v>
       </c>
-      <c r="F5" s="48">
+      <c r="F5" s="46">
         <v>46383</v>
       </c>
     </row>
     <row r="6" ht="12" customHeight="1" spans="1:6">
-      <c r="A6" s="46"/>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="46"/>
-      <c r="E6" s="48"/>
-      <c r="F6" s="46"/>
+      <c r="A6" s="44"/>
+      <c r="B6" s="44"/>
+      <c r="C6" s="44"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="44"/>
     </row>
     <row r="7" ht="12" customHeight="1" spans="1:6">
-      <c r="A7" s="46"/>
-      <c r="B7" s="46"/>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="48"/>
-      <c r="F7" s="46"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="46"/>
+      <c r="F7" s="44"/>
     </row>
     <row r="8" ht="12" customHeight="1" spans="1:6">
-      <c r="A8" s="46"/>
-      <c r="B8" s="46"/>
-      <c r="C8" s="46"/>
-      <c r="D8" s="46"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="46"/>
-    </row>
-    <row r="9" s="43" customFormat="1" ht="12" customHeight="1" spans="1:6">
-      <c r="A9" s="50"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="48"/>
-      <c r="F9" s="50"/>
-    </row>
-    <row r="10" s="43" customFormat="1" ht="12" customHeight="1" spans="1:6">
-      <c r="A10" s="50"/>
-      <c r="B10" s="50"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="50"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="50"/>
+      <c r="A8" s="44"/>
+      <c r="B8" s="44"/>
+      <c r="C8" s="44"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="46"/>
+      <c r="F8" s="44"/>
+    </row>
+    <row r="9" s="41" customFormat="1" ht="12" customHeight="1" spans="1:6">
+      <c r="A9" s="48"/>
+      <c r="B9" s="48"/>
+      <c r="C9" s="48"/>
+      <c r="D9" s="48"/>
+      <c r="E9" s="46"/>
+      <c r="F9" s="48"/>
+    </row>
+    <row r="10" s="41" customFormat="1" ht="12" customHeight="1" spans="1:6">
+      <c r="A10" s="48"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2149,406 +2138,406 @@
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1" spans="1:7">
-      <c r="B1" s="16" t="s">
+      <c r="B1" s="14" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="2" ht="12.75" customHeight="1" spans="1:7">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="17"/>
+      <c r="A2" s="15"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="15"/>
     </row>
     <row r="3" ht="12.75" customHeight="1" spans="1:7">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="19" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="4" ht="12.75" customHeight="1" spans="1:7">
-      <c r="A4" s="22"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="23"/>
+      <c r="A4" s="20"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="21"/>
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:7">
-      <c r="A5" s="24"/>
-      <c r="B5" s="25" t="s">
+      <c r="A5" s="22"/>
+      <c r="B5" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C5" s="26"/>
+      <c r="C5" s="24"/>
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:7">
-      <c r="A6" s="27">
+      <c r="A6" s="25">
         <v>1</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="27">
+      <c r="C6" s="25">
         <v>2</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:7">
-      <c r="A7" s="28">
+      <c r="A7" s="26">
         <v>2</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C7" s="29">
+      <c r="C7" s="27">
         <v>3</v>
       </c>
-      <c r="G7" s="30"/>
+      <c r="G7" s="28"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:7">
-      <c r="A8" s="28">
+      <c r="A8" s="26">
         <v>3</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:7">
-      <c r="A9" s="28">
+      <c r="A9" s="26">
         <v>4</v>
       </c>
-      <c r="B9" s="31" t="s">
+      <c r="B9" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="29">
+      <c r="C9" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:7">
-      <c r="A10" s="28">
+      <c r="A10" s="26">
         <v>5</v>
       </c>
-      <c r="B10" s="31" t="s">
+      <c r="B10" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:7">
-      <c r="A11" s="28">
+      <c r="A11" s="26">
         <v>6</v>
       </c>
-      <c r="B11" s="31" t="s">
+      <c r="B11" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="29">
+      <c r="C11" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:7">
-      <c r="A12" s="28">
+      <c r="A12" s="26">
         <v>7</v>
       </c>
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:7">
-      <c r="A13" s="28">
+      <c r="A13" s="26">
         <v>8</v>
       </c>
-      <c r="B13" s="31" t="s">
+      <c r="B13" s="29" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="29">
+      <c r="C13" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:7">
-      <c r="A14" s="28">
+      <c r="A14" s="26">
         <v>9</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:7">
-      <c r="A15" s="28">
+      <c r="A15" s="26">
         <v>10</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:7">
-      <c r="A16" s="28">
+      <c r="A16" s="26">
         <v>11</v>
       </c>
-      <c r="B16" s="31" t="s">
+      <c r="B16" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:3">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25" t="s">
+      <c r="A17" s="22"/>
+      <c r="B17" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="26"/>
+      <c r="C17" s="24"/>
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:3">
-      <c r="A18" s="28">
+      <c r="A18" s="26">
         <v>12</v>
       </c>
-      <c r="B18" s="32" t="s">
+      <c r="B18" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C18" s="29">
+      <c r="C18" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:3">
-      <c r="A19" s="28">
+      <c r="A19" s="26">
         <v>13</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B19" s="29" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:3">
-      <c r="A20" s="28">
+      <c r="A20" s="26">
         <v>14</v>
       </c>
-      <c r="B20" s="31" t="s">
+      <c r="B20" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="C20" s="29">
+      <c r="C20" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:3">
-      <c r="A21" s="28">
+      <c r="A21" s="26">
         <v>15</v>
       </c>
-      <c r="B21" s="31" t="s">
+      <c r="B21" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="29">
+      <c r="C21" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:3">
-      <c r="A22" s="28">
+      <c r="A22" s="26">
         <v>16</v>
       </c>
-      <c r="B22" s="31" t="s">
+      <c r="B22" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="29">
+      <c r="C22" s="27">
         <v>2</v>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:3">
-      <c r="A23" s="28"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="29"/>
+      <c r="A23" s="26"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="27"/>
     </row>
     <row r="24" ht="15" customHeight="1" spans="1:3">
-      <c r="A24" s="24"/>
-      <c r="B24" s="25" t="s">
+      <c r="A24" s="22"/>
+      <c r="B24" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="C24" s="26"/>
+      <c r="C24" s="24"/>
     </row>
     <row r="25" ht="15" customHeight="1" spans="1:3">
-      <c r="A25" s="28">
+      <c r="A25" s="26">
         <v>17</v>
       </c>
-      <c r="B25" s="32" t="s">
+      <c r="B25" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" spans="1:3">
-      <c r="A26" s="28">
+      <c r="A26" s="26">
         <v>18</v>
       </c>
-      <c r="B26" s="31" t="s">
+      <c r="B26" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="C26" s="29">
+      <c r="C26" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" spans="1:3">
-      <c r="A27" s="28">
+      <c r="A27" s="26">
         <v>19</v>
       </c>
-      <c r="B27" s="31" t="s">
+      <c r="B27" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" spans="1:3">
-      <c r="A28" s="28">
+      <c r="A28" s="26">
         <v>20</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="30" t="s">
         <v>41</v>
       </c>
-      <c r="C28" s="29">
+      <c r="C28" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" spans="1:3">
-      <c r="A29" s="28">
+      <c r="A29" s="26">
         <v>21</v>
       </c>
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="C29" s="29">
+      <c r="C29" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" spans="1:3">
-      <c r="A30" s="28">
+      <c r="A30" s="26">
         <v>22</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="30" t="s">
         <v>43</v>
       </c>
-      <c r="C30" s="29">
+      <c r="C30" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" spans="1:3">
-      <c r="A31" s="28">
+      <c r="A31" s="26">
         <v>23</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="C31" s="29">
+      <c r="C31" s="27">
         <v>3</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" spans="1:3">
-      <c r="A32" s="28">
+      <c r="A32" s="26">
         <v>24</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="29" t="s">
         <v>45</v>
       </c>
-      <c r="C32" s="29">
+      <c r="C32" s="27">
         <v>8</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" spans="1:3">
-      <c r="A33" s="24"/>
-      <c r="B33" s="25" t="s">
+      <c r="A33" s="22"/>
+      <c r="B33" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="C33" s="26"/>
+      <c r="C33" s="24"/>
     </row>
     <row r="34" ht="15" customHeight="1" spans="1:3">
-      <c r="A34" s="28">
+      <c r="A34" s="26">
         <v>25</v>
       </c>
-      <c r="B34" s="32" t="s">
+      <c r="B34" s="30" t="s">
         <v>47</v>
       </c>
-      <c r="C34" s="29">
+      <c r="C34" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" spans="1:3">
-      <c r="A35" s="28">
+      <c r="A35" s="26">
         <v>26</v>
       </c>
-      <c r="B35" s="31" t="s">
+      <c r="B35" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="29">
+      <c r="C35" s="27">
         <v>5</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" spans="1:3">
-      <c r="A36" s="33"/>
-      <c r="B36" s="34" t="s">
+      <c r="A36" s="31"/>
+      <c r="B36" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="C36" s="35"/>
+      <c r="C36" s="33"/>
     </row>
     <row r="37" ht="15" customHeight="1" spans="1:3">
-      <c r="A37" s="36">
+      <c r="A37" s="34">
         <v>27</v>
       </c>
-      <c r="B37" s="37" t="s">
+      <c r="B37" s="35" t="s">
         <v>50</v>
       </c>
-      <c r="C37" s="38">
+      <c r="C37" s="36">
         <v>8</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" spans="1:3">
-      <c r="A38" s="36">
+      <c r="A38" s="34">
         <v>28</v>
       </c>
-      <c r="B38" s="39" t="s">
+      <c r="B38" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C38" s="38">
+      <c r="C38" s="36">
         <v>5</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" spans="1:3">
-      <c r="A39" s="40">
+      <c r="A39" s="38">
         <v>29</v>
       </c>
-      <c r="B39" s="41" t="s">
+      <c r="B39" s="39" t="s">
         <v>52</v>
       </c>
-      <c r="C39" s="42">
+      <c r="C39" s="40">
         <v>8</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" spans="1:3">
-      <c r="A40" s="36">
+      <c r="A40" s="34">
         <v>30</v>
       </c>
-      <c r="B40" s="37" t="s">
+      <c r="B40" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="C40" s="38">
+      <c r="C40" s="36">
         <v>8</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" spans="1:3">
-      <c r="A41" s="27"/>
-      <c r="B41" s="27"/>
-      <c r="C41" s="27"/>
+      <c r="A41" s="25"/>
+      <c r="B41" s="25"/>
+      <c r="C41" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2582,1006 +2571,1040 @@
       </c>
     </row>
     <row r="2" ht="18" customHeight="1" spans="1:10">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
     </row>
     <row r="3" ht="12.75" customHeight="1" spans="1:10">
-      <c r="B3" s="4"/>
-      <c r="E3" s="5"/>
-      <c r="G3" s="5"/>
+      <c r="B3" s="3"/>
+      <c r="E3" s="4"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="H4" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="I4" s="6" t="s">
+      <c r="I4" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="J4" s="6" t="s">
+      <c r="J4" s="5" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="5" ht="12" customHeight="1" spans="1:10">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6">
         <f>SUM(C7:C41)</f>
         <v>121</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
     </row>
     <row r="6" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="9"/>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="9"/>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="10"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="8"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:10">
-      <c r="A7" s="11">
+      <c r="A7" s="10">
         <v>1</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="11">
+      <c r="C7" s="10">
         <v>2</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="12">
         <v>46279</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="12">
         <v>46286</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="12">
         <v>46288</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H7" s="12">
         <v>46302</v>
       </c>
-      <c r="I7" s="11">
+      <c r="I7" s="10">
         <v>2</v>
       </c>
-      <c r="J7" s="12" t="s">
+      <c r="J7" s="11" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:10">
-      <c r="A8" s="11">
+      <c r="A8" s="10">
         <v>17</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="11">
+      <c r="C8" s="10">
         <v>5</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="12">
         <v>46279</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="12">
         <v>46286</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="12">
         <v>46288</v>
       </c>
-      <c r="H8" s="13">
+      <c r="H8" s="12">
         <v>46302</v>
       </c>
-      <c r="I8" s="11">
+      <c r="I8" s="10">
         <v>5</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="J8" s="11" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:10">
-      <c r="A9" s="11">
+      <c r="A9" s="10">
         <v>19</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="11">
+      <c r="C9" s="10">
         <v>5</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="12">
         <v>46279</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="12">
         <v>46286</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="12">
         <v>46288</v>
       </c>
-      <c r="H9" s="13">
+      <c r="H9" s="12">
         <v>46302</v>
       </c>
-      <c r="I9" s="11">
+      <c r="I9" s="10">
         <v>5</v>
       </c>
-      <c r="J9" s="12" t="s">
+      <c r="J9" s="11" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:10">
-      <c r="A10" s="11">
+      <c r="A10" s="10">
         <v>2</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="11">
+      <c r="C10" s="10">
         <v>3</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="12">
         <v>46279</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="12">
         <v>46286</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="12">
         <v>46289</v>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="12">
         <v>46302</v>
       </c>
-      <c r="I10" s="11">
+      <c r="I10" s="10">
         <v>3</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="11" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:10">
-      <c r="A11" s="11">
+      <c r="A11" s="10">
         <v>3</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="11">
+      <c r="C11" s="10">
         <v>2</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="12">
         <v>46279</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="12">
         <v>46286</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="12">
         <v>46289</v>
       </c>
-      <c r="H11" s="13">
+      <c r="H11" s="12">
         <v>46302</v>
       </c>
-      <c r="I11" s="11">
+      <c r="I11" s="10">
         <v>2</v>
       </c>
-      <c r="J11" s="12" t="s">
+      <c r="J11" s="11" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:10">
-      <c r="A12" s="11">
+      <c r="A12" s="10">
         <v>4</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="11">
+      <c r="C12" s="10">
         <v>3</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="12">
         <v>46279</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="12">
         <v>46286</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="12">
         <v>46289</v>
       </c>
-      <c r="H12" s="13">
+      <c r="H12" s="12">
         <v>46302</v>
       </c>
-      <c r="I12" s="11">
+      <c r="I12" s="10">
         <v>3</v>
       </c>
-      <c r="J12" s="12" t="s">
+      <c r="J12" s="11" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:10">
-      <c r="A13" s="11">
+      <c r="A13" s="10">
         <v>18</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="11">
+      <c r="C13" s="10">
         <v>3</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="13">
+      <c r="E13" s="12">
         <v>46279</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="12">
         <v>46286</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="12">
         <v>46289</v>
       </c>
-      <c r="H13" s="13">
+      <c r="H13" s="12">
         <v>46302</v>
       </c>
-      <c r="I13" s="11">
+      <c r="I13" s="10">
         <v>3</v>
       </c>
-      <c r="J13" s="12" t="s">
+      <c r="J13" s="11" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="14" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="10"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="9"/>
     </row>
     <row r="15" ht="12" customHeight="1" spans="1:10">
-      <c r="A15" s="11">
+      <c r="A15" s="10">
         <v>5</v>
       </c>
-      <c r="B15" s="14" t="s">
+      <c r="B15" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C15" s="11">
+      <c r="C15" s="10">
         <v>2</v>
       </c>
-      <c r="D15" s="14" t="s">
+      <c r="D15" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="12">
         <v>46316</v>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="12">
         <v>46327</v>
       </c>
-      <c r="G15" s="13">
+      <c r="G15" s="12">
         <v>46317</v>
       </c>
-      <c r="H15" s="13">
+      <c r="H15" s="12">
         <v>46317</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I15" s="10">
         <v>2</v>
       </c>
-      <c r="J15" s="14" t="s">
+      <c r="J15" s="11" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="16" ht="12" customHeight="1" spans="1:10">
-      <c r="A16" s="11">
+      <c r="A16" s="10">
         <v>27</v>
       </c>
-      <c r="B16" s="14" t="s">
+      <c r="B16" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="C16" s="11">
+      <c r="C16" s="10">
         <v>8</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="12">
         <v>46316</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="12">
         <v>46327</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="12">
         <v>46316</v>
       </c>
-      <c r="H16" s="13">
+      <c r="H16" s="12">
         <v>46316</v>
       </c>
-      <c r="I16" s="11">
+      <c r="I16" s="10">
         <v>8</v>
       </c>
-      <c r="J16" s="14" t="s">
+      <c r="J16" s="11" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="17" ht="12" customHeight="1" spans="1:10">
-      <c r="A17" s="11">
+      <c r="A17" s="10">
         <v>28</v>
       </c>
-      <c r="B17" s="14" t="s">
+      <c r="B17" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="10">
         <v>5</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="12">
         <v>46316</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F17" s="12">
         <v>46327</v>
       </c>
-      <c r="G17" s="13">
+      <c r="G17" s="12">
         <v>46316</v>
       </c>
-      <c r="H17" s="13">
+      <c r="H17" s="12">
         <v>46316</v>
       </c>
-      <c r="I17" s="11">
+      <c r="I17" s="10">
         <v>5</v>
       </c>
-      <c r="J17" s="14" t="s">
+      <c r="J17" s="11" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="18" ht="12" customHeight="1" spans="1:10">
-      <c r="A18" s="11">
+      <c r="A18" s="10">
         <v>25</v>
       </c>
-      <c r="B18" s="14" t="s">
+      <c r="B18" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="10">
         <v>5</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E18" s="13">
+      <c r="E18" s="12">
         <v>46316</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="12">
         <v>46327</v>
       </c>
-      <c r="G18" s="13">
+      <c r="G18" s="12">
         <v>46322</v>
       </c>
-      <c r="H18" s="13">
+      <c r="H18" s="12">
         <v>46322</v>
       </c>
-      <c r="I18" s="11">
+      <c r="I18" s="10">
         <v>5</v>
       </c>
-      <c r="J18" s="14" t="s">
+      <c r="J18" s="11" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="19" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A19" s="15" t="s">
+      <c r="A19" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
     </row>
     <row r="20" ht="12" customHeight="1" spans="1:10">
-      <c r="A20" s="11">
+      <c r="A20" s="10">
         <v>7</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="B20" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="10">
         <v>5</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E20" s="13">
+      <c r="E20" s="12">
         <v>46328</v>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="12">
         <v>46341</v>
       </c>
-      <c r="G20" s="13">
+      <c r="G20" s="12">
         <v>46323</v>
       </c>
-      <c r="H20" s="13">
+      <c r="H20" s="12">
         <v>46323</v>
       </c>
-      <c r="I20" s="11">
+      <c r="I20" s="10">
         <v>5</v>
       </c>
-      <c r="J20" s="14" t="s">
+      <c r="J20" s="11" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="21" ht="12" customHeight="1" spans="1:10">
-      <c r="A21" s="11">
+      <c r="A21" s="10">
         <v>8</v>
       </c>
-      <c r="B21" s="14" t="s">
+      <c r="B21" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <v>3</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="13">
+      <c r="E21" s="12">
         <v>46328</v>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="12">
         <v>46341</v>
       </c>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="11"/>
-      <c r="J21" s="14" t="s">
+      <c r="G21" s="12">
+        <v>46325.0000106713</v>
+      </c>
+      <c r="H21" s="12">
+        <v>46325.0000106713</v>
+      </c>
+      <c r="I21" s="10">
+        <v>3</v>
+      </c>
+      <c r="J21" s="11" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="22" ht="12" customHeight="1" spans="1:10">
-      <c r="A22" s="11">
+      <c r="A22" s="10">
         <v>21</v>
       </c>
-      <c r="B22" s="14" t="s">
+      <c r="B22" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="10">
         <v>5</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="12">
         <v>46328</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="12">
         <v>46341</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="12">
         <v>46323</v>
       </c>
-      <c r="H22" s="13">
+      <c r="H22" s="12">
         <v>46323</v>
       </c>
-      <c r="I22" s="11">
+      <c r="I22" s="10">
         <v>5</v>
       </c>
-      <c r="J22" s="14" t="s">
+      <c r="J22" s="11" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="23" ht="12" customHeight="1" spans="1:10">
-      <c r="A23" s="11">
+      <c r="A23" s="10">
         <v>26</v>
       </c>
-      <c r="B23" s="14" t="s">
+      <c r="B23" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="10">
         <v>5</v>
       </c>
-      <c r="D23" s="14" t="s">
+      <c r="D23" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="12">
         <v>46328</v>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="12">
         <v>46341</v>
       </c>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="11"/>
-      <c r="J23" s="14" t="s">
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="10"/>
+      <c r="J23" s="11" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="24" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="9"/>
-      <c r="H24" s="9"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
     </row>
     <row r="25" ht="12" customHeight="1" spans="1:10">
-      <c r="A25" s="11">
+      <c r="A25" s="10">
         <v>10</v>
       </c>
-      <c r="B25" s="14" t="s">
+      <c r="B25" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="10">
         <v>5</v>
       </c>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E25" s="13">
+      <c r="E25" s="12">
         <v>46342</v>
       </c>
-      <c r="F25" s="13">
+      <c r="F25" s="12">
         <v>46355</v>
       </c>
-      <c r="G25" s="13"/>
-      <c r="H25" s="13"/>
-      <c r="I25" s="11"/>
-      <c r="J25" s="14" t="s">
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="11" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="26" ht="12" customHeight="1" spans="1:10">
-      <c r="A26" s="11">
+      <c r="A26" s="10">
         <v>11</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="B26" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="10">
         <v>3</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="12">
         <v>46342</v>
       </c>
-      <c r="F26" s="13">
+      <c r="F26" s="12">
         <v>46355</v>
       </c>
-      <c r="G26" s="13"/>
-      <c r="H26" s="13"/>
-      <c r="I26" s="11"/>
-      <c r="J26" s="14" t="s">
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="10"/>
+      <c r="J26" s="11" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="27" ht="12" customHeight="1" spans="1:10">
-      <c r="A27" s="11">
+      <c r="A27" s="10">
         <v>22</v>
       </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="10">
         <v>5</v>
       </c>
-      <c r="D27" s="14" t="s">
+      <c r="D27" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E27" s="13">
+      <c r="E27" s="12">
         <v>46342</v>
       </c>
-      <c r="F27" s="13">
+      <c r="F27" s="12">
         <v>46355</v>
       </c>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="11"/>
-      <c r="J27" s="14" t="s">
+      <c r="G27" s="12">
+        <v>46325.0000018171</v>
+      </c>
+      <c r="H27" s="12">
+        <v>46325.0000018171</v>
+      </c>
+      <c r="I27" s="10">
+        <v>5</v>
+      </c>
+      <c r="J27" s="11" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="28" ht="12" customHeight="1" spans="1:10">
-      <c r="A28" s="11">
+      <c r="A28" s="10">
         <v>23</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="10">
         <v>3</v>
       </c>
-      <c r="D28" s="14" t="s">
+      <c r="D28" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E28" s="13">
+      <c r="E28" s="12">
         <v>46342</v>
       </c>
-      <c r="F28" s="13">
+      <c r="F28" s="12">
         <v>46355</v>
       </c>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="11"/>
-      <c r="J28" s="14" t="s">
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+      <c r="I28" s="10"/>
+      <c r="J28" s="11" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="29" ht="12" customHeight="1" spans="1:10">
-      <c r="A29" s="11">
+      <c r="A29" s="10">
         <v>24</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B29" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="10">
         <v>8</v>
       </c>
-      <c r="D29" s="14" t="s">
+      <c r="D29" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E29" s="13">
+      <c r="E29" s="12">
         <v>46342</v>
       </c>
-      <c r="F29" s="13">
+      <c r="F29" s="12">
         <v>46355</v>
       </c>
-      <c r="G29" s="13"/>
-      <c r="H29" s="13"/>
-      <c r="I29" s="11"/>
-      <c r="J29" s="14" t="s">
+      <c r="G29" s="12">
+        <v>46325.0000044676</v>
+      </c>
+      <c r="H29" s="12">
+        <v>46325.0000044676</v>
+      </c>
+      <c r="I29" s="10">
+        <v>8</v>
+      </c>
+      <c r="J29" s="11" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="30" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="B30" s="9"/>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="9"/>
-      <c r="F30" s="9"/>
-      <c r="G30" s="9"/>
-      <c r="H30" s="9"/>
-      <c r="I30" s="9"/>
-      <c r="J30" s="9"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
+      <c r="H30" s="8"/>
+      <c r="I30" s="8"/>
+      <c r="J30" s="8"/>
     </row>
     <row r="31" ht="12" customHeight="1" spans="1:10">
-      <c r="A31" s="11">
+      <c r="A31" s="10">
         <v>6</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="10">
         <v>3</v>
       </c>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E31" s="13">
+      <c r="E31" s="12">
         <v>46356</v>
       </c>
-      <c r="F31" s="13">
+      <c r="F31" s="12">
         <v>46369</v>
       </c>
-      <c r="G31" s="13"/>
-      <c r="H31" s="13"/>
-      <c r="I31" s="11"/>
-      <c r="J31" s="14" t="s">
-        <v>89</v>
+      <c r="G31" s="12" t="d">
+        <v>2026-10-31T00:00:00.000Z</v>
+      </c>
+      <c r="H31" s="12"/>
+      <c r="I31" s="10"/>
+      <c r="J31" s="11" t="str">
+        <v>Code hoàn thành trên codex/s5-us06-reminders (52554fd), đã test tích hợp trên codex/s5-phu-integration (118/118 API tests, Web build). Chờ review/merge main; US-26 cấu hình lịch nhắc do Kiệt đang chờ.</v>
       </c>
     </row>
     <row r="32" ht="12" customHeight="1" spans="1:10">
-      <c r="A32" s="11">
+      <c r="A32" s="10">
         <v>9</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="10">
         <v>3</v>
       </c>
-      <c r="D32" s="14" t="s">
+      <c r="D32" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E32" s="13">
+      <c r="E32" s="12">
         <v>46356</v>
       </c>
-      <c r="F32" s="13">
+      <c r="F32" s="12">
         <v>46369</v>
       </c>
-      <c r="G32" s="13"/>
-      <c r="H32" s="13"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="14" t="s">
-        <v>90</v>
+      <c r="G32" s="12" t="d">
+        <v>2026-10-30T00:00:00.000Z</v>
+      </c>
+      <c r="H32" s="12" t="d">
+        <v>2026-10-30T00:00:00.000Z</v>
+      </c>
+      <c r="I32" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="11" t="str">
+        <v>Done (merge main 30/10): API + Web không gian trao đổi lớp; phân quyền theo lớp và integration tests (42f8fc8).</v>
       </c>
     </row>
     <row r="33" ht="12" customHeight="1" spans="1:10">
-      <c r="A33" s="11">
+      <c r="A33" s="10">
         <v>12</v>
       </c>
-      <c r="B33" s="14" t="s">
+      <c r="B33" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <v>2</v>
       </c>
-      <c r="D33" s="14" t="s">
+      <c r="D33" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E33" s="13">
+      <c r="E33" s="12">
         <v>46356</v>
       </c>
-      <c r="F33" s="13">
+      <c r="F33" s="12">
         <v>46369</v>
       </c>
-      <c r="G33" s="13"/>
-      <c r="H33" s="13"/>
-      <c r="I33" s="11"/>
-      <c r="J33" s="14" t="s">
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="10"/>
+      <c r="J33" s="11" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="34" ht="12" customHeight="1" spans="1:10">
-      <c r="A34" s="11">
+      <c r="A34" s="10">
         <v>13</v>
       </c>
-      <c r="B34" s="14" t="s">
+      <c r="B34" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C34" s="11">
+      <c r="C34" s="10">
         <v>2</v>
       </c>
-      <c r="D34" s="14" t="s">
+      <c r="D34" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E34" s="13">
+      <c r="E34" s="12">
         <v>46356</v>
       </c>
-      <c r="F34" s="13">
+      <c r="F34" s="12">
         <v>46369</v>
       </c>
-      <c r="G34" s="13"/>
-      <c r="H34" s="13"/>
-      <c r="I34" s="11"/>
-      <c r="J34" s="14" t="s">
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="10"/>
+      <c r="J34" s="11" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="35" ht="12" customHeight="1" spans="1:10">
-      <c r="A35" s="11">
+      <c r="A35" s="10">
         <v>14</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="11">
+      <c r="C35" s="10">
         <v>3</v>
       </c>
-      <c r="D35" s="14" t="s">
+      <c r="D35" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E35" s="13">
+      <c r="E35" s="12">
         <v>46356</v>
       </c>
-      <c r="F35" s="13">
+      <c r="F35" s="12">
         <v>46369</v>
       </c>
-      <c r="G35" s="13"/>
-      <c r="H35" s="13"/>
-      <c r="I35" s="11"/>
-      <c r="J35" s="14" t="s">
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="10"/>
+      <c r="J35" s="11" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="36" ht="12" customHeight="1" spans="1:10">
-      <c r="A36" s="11">
+      <c r="A36" s="10">
         <v>15</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="11">
+      <c r="C36" s="10">
         <v>2</v>
       </c>
-      <c r="D36" s="14" t="s">
+      <c r="D36" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E36" s="13">
+      <c r="E36" s="12">
         <v>46356</v>
       </c>
-      <c r="F36" s="13">
+      <c r="F36" s="12">
         <v>46369</v>
       </c>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="11"/>
-      <c r="J36" s="14" t="s">
-        <v>94</v>
+      <c r="G36" s="12" t="d">
+        <v>2026-10-30T00:00:00.000Z</v>
+      </c>
+      <c r="H36" s="12" t="d">
+        <v>2026-10-30T00:00:00.000Z</v>
+      </c>
+      <c r="I36" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J36" s="11" t="str">
+        <v>Done (merge main 30/10): lớp trưởng chuyển câu hỏi lên Phòng QL HSSV, chống Pending trùng và rút lại; API + Web + tests (4c846ca).</v>
       </c>
     </row>
     <row r="37" ht="12" customHeight="1" spans="1:10">
-      <c r="A37" s="11">
+      <c r="A37" s="10">
         <v>16</v>
       </c>
-      <c r="B37" s="14" t="s">
+      <c r="B37" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C37" s="11">
+      <c r="C37" s="10">
         <v>2</v>
       </c>
-      <c r="D37" s="14" t="s">
+      <c r="D37" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E37" s="13">
+      <c r="E37" s="12">
         <v>46356</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="12">
         <v>46369</v>
       </c>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="11"/>
-      <c r="J37" s="14" t="s">
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="10"/>
+      <c r="J37" s="11" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="38" ht="12" customHeight="1" spans="1:10">
-      <c r="A38" s="11">
+      <c r="A38" s="10">
         <v>20</v>
       </c>
-      <c r="B38" s="14" t="s">
+      <c r="B38" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="C38" s="11">
+      <c r="C38" s="10">
         <v>3</v>
       </c>
-      <c r="D38" s="14" t="s">
+      <c r="D38" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E38" s="13">
+      <c r="E38" s="12">
         <v>46356</v>
       </c>
-      <c r="F38" s="13">
+      <c r="F38" s="12">
         <v>46369</v>
       </c>
-      <c r="G38" s="13"/>
-      <c r="H38" s="13"/>
-      <c r="I38" s="11"/>
-      <c r="J38" s="14" t="s">
-        <v>96</v>
+      <c r="G38" s="12" t="d">
+        <v>2026-10-31T00:00:00.000Z</v>
+      </c>
+      <c r="H38" s="12"/>
+      <c r="I38" s="10"/>
+      <c r="J38" s="11" t="str">
+        <v>Code hoàn thành trên codex/s5-us20-staff-escalations (707da1b), đã test tích hợp trên codex/s5-phu-integration (118/118 API tests, Web build). Chờ review/merge main; US-16 relay về lớp do Kiệt làm.</v>
       </c>
     </row>
     <row r="39" ht="12.75" customHeight="1" spans="1:10">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="13" t="s">
         <v>97</v>
       </c>
-      <c r="B39" s="9"/>
-      <c r="C39" s="9"/>
-      <c r="D39" s="9"/>
-      <c r="E39" s="9"/>
-      <c r="F39" s="9"/>
-      <c r="G39" s="9"/>
-      <c r="H39" s="9"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
+      <c r="H39" s="8"/>
+      <c r="I39" s="8"/>
+      <c r="J39" s="8"/>
     </row>
     <row r="40" ht="12" customHeight="1" spans="1:10">
-      <c r="A40" s="11">
+      <c r="A40" s="10">
         <v>29</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="11">
+      <c r="C40" s="10">
         <v>8</v>
       </c>
-      <c r="D40" s="14" t="s">
+      <c r="D40" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E40" s="13">
+      <c r="E40" s="12">
         <v>46370</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="12">
         <v>46383</v>
       </c>
-      <c r="G40" s="13"/>
-      <c r="H40" s="13"/>
-      <c r="I40" s="11"/>
-      <c r="J40" s="14" t="s">
+      <c r="G40" s="12"/>
+      <c r="H40" s="12"/>
+      <c r="I40" s="10"/>
+      <c r="J40" s="11" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="41" ht="12" customHeight="1" spans="1:10">
-      <c r="A41" s="11">
+      <c r="A41" s="10">
         <v>30</v>
       </c>
-      <c r="B41" s="14" t="s">
+      <c r="B41" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="C41" s="11">
+      <c r="C41" s="10">
         <v>8</v>
       </c>
-      <c r="D41" s="14" t="s">
+      <c r="D41" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="E41" s="13">
+      <c r="E41" s="12">
         <v>46370</v>
       </c>
-      <c r="F41" s="13">
+      <c r="F41" s="12">
         <v>46383</v>
       </c>
-      <c r="G41" s="13"/>
-      <c r="H41" s="13"/>
-      <c r="I41" s="11"/>
-      <c r="J41" s="14" t="s">
+      <c r="G41" s="12"/>
+      <c r="H41" s="12"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="11" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(backlog): refresh Sprint 5 verification count
</commit_message>
<xml_diff>
--- a/Nhom8_ProductBacklog.xlsx
+++ b/Nhom8_ProductBacklog.xlsx
@@ -3343,7 +3343,7 @@
       <c r="H31" s="12"/>
       <c r="I31" s="10"/>
       <c r="J31" s="11" t="str">
-        <v>Code hoàn thành trên codex/s5-us06-reminders (52554fd), đã test tích hợp trên codex/s5-phu-integration (118/118 API tests, Web build). Chờ review/merge main; US-26 cấu hình lịch nhắc do Kiệt đang chờ.</v>
+        <v>Code hoàn thành trên codex/s5-us06-reminders (52554fd), đã test tích hợp trên codex/s5-phu-integration (119/119 API tests, Web build). Chờ review/merge main; US-26 cấu hình lịch nhắc do Kiệt đang chờ.</v>
       </c>
     </row>
     <row r="32" ht="12" customHeight="1" spans="1:10">
@@ -3539,7 +3539,7 @@
       <c r="H38" s="12"/>
       <c r="I38" s="10"/>
       <c r="J38" s="11" t="str">
-        <v>Code hoàn thành trên codex/s5-us20-staff-escalations (707da1b), đã test tích hợp trên codex/s5-phu-integration (118/118 API tests, Web build). Chờ review/merge main; US-16 relay về lớp do Kiệt làm.</v>
+        <v>Code hoàn thành trên codex/s5-us20-staff-escalations (707da1b), đã test tích hợp trên codex/s5-phu-integration (119/119 API tests, Web build). Chờ review/merge main; US-16 relay về lớp do Kiệt làm.</v>
       </c>
     </row>
     <row r="39" ht="12.75" customHeight="1" spans="1:10">

</xml_diff>